<commit_message>
Add translation comparison script and LLM translation functionality
- Introduced `compare_translate.py` for comparing Google Translate and Gemini translations on a set of sentences.
- Added `llm_translate.py` for English to Vietnamese translation using Gemini LLM, replacing Google Translate.
- Updated Excel files for translation comparison results.
- Implemented error handling and model selection for API requests.
</commit_message>
<xml_diff>
--- a/data/Noi dung SICK/00 MUC LUC.xlsx
+++ b/data/Noi dung SICK/00 MUC LUC.xlsx
@@ -748,7 +748,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Đầu đọc RFID</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Đầu đọc RFID</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Đầu đọc RFID</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3178,11 +3178,7 @@
       <c r="F74" t="n">
         <v>0</v>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>Thiết bị phân tích khí và bụi</t>
-        </is>
-      </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/analyzers/air-quality-measuring-devices/c/g407184</t>
@@ -3216,11 +3212,7 @@
       <c r="F75" t="n">
         <v>0</v>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>Thiết bị phân tích khí và bụi</t>
-        </is>
-      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/analyzers/digital-analyzer-solutions/c/g284256</t>
@@ -3254,11 +3246,7 @@
       <c r="F76" t="n">
         <v>0</v>
       </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Thiết bị phân tích khí và bụi</t>
-        </is>
-      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/analyzers/dust-measuring-devices/c/g54727</t>
@@ -3292,11 +3280,7 @@
       <c r="F77" t="n">
         <v>0</v>
       </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>Thiết bị phân tích khí và bụi</t>
-        </is>
-      </c>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/analyzers/gas-analyzers/c/g54724</t>
@@ -3330,11 +3314,7 @@
       <c r="F78" t="n">
         <v>0</v>
       </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Thiết bị phân tích khí và bụi</t>
-        </is>
-      </c>
+      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/analyzers/smoke-detectors/c/g284260</t>
@@ -3368,11 +3348,7 @@
       <c r="F79" t="n">
         <v>0</v>
       </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Thiết bị phân tích khí và bụi</t>
-        </is>
-      </c>
+      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/analyzers/visual-range-measuring-devices/c/g284262</t>
@@ -6408,11 +6384,7 @@
       <c r="F159" t="n">
         <v>56</v>
       </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>Cảm biến công nghiệp, Cảm biến tiệm cận</t>
-        </is>
-      </c>
+      <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/detection-sensors/inductive-proximity-sensors/imx/c/g555781</t>
@@ -7700,11 +7672,7 @@
       <c r="F193" t="n">
         <v>274</v>
       </c>
-      <c r="G193" t="inlineStr">
-        <is>
-          <t>Cảm biến công nghiệp, Cảm biến quang điện</t>
-        </is>
-      </c>
+      <c r="G193" t="inlineStr"/>
       <c r="H193" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/detection-sensors/photoelectric-sensors/w100/c/g184875</t>
@@ -8080,11 +8048,7 @@
       <c r="F203" t="n">
         <v>78</v>
       </c>
-      <c r="G203" t="inlineStr">
-        <is>
-          <t>Cảm biến công nghiệp, Cảm biến quang điện</t>
-        </is>
-      </c>
+      <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/detection-sensors/photoelectric-sensors/w250/c/g203757</t>
@@ -8194,11 +8158,7 @@
       <c r="F206" t="n">
         <v>62</v>
       </c>
-      <c r="G206" t="inlineStr">
-        <is>
-          <t>Cảm biến công nghiệp, Cảm biến quang điện</t>
-        </is>
-      </c>
+      <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/detection-sensors/photoelectric-sensors/w280/c/g204129</t>
@@ -9260,7 +9220,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>Cảm biến công nghiệp, Cảm biến quang điện</t>
+          <t>Cảm biến công nghiệp, Cảm biến đo khoảng cách</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -9298,7 +9258,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Cảm biến công nghiệp, Cảm biến quang điện</t>
+          <t>Cảm biến công nghiệp, Cảm biến đo khoảng cách</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -9336,7 +9296,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Cảm biến công nghiệp, Cảm biến quang điện</t>
+          <t>Cảm biến công nghiệp, Cảm biến đo khoảng cách</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -9374,7 +9334,7 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Cảm biến công nghiệp, Cảm biến quang điện</t>
+          <t>Cảm biến công nghiệp, Cảm biến đo khoảng cách</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
@@ -9412,7 +9372,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Cảm biến công nghiệp, Cảm biến quang điện</t>
+          <t>Cảm biến công nghiệp, Cảm biến đo khoảng cách</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -9714,11 +9674,7 @@
       <c r="F246" t="n">
         <v>0</v>
       </c>
-      <c r="G246" t="inlineStr">
-        <is>
-          <t>Cảm biến công nghiệp, Cảm biến lưu lượng</t>
-        </is>
-      </c>
+      <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/flow-measurement/digital-flow-solutions/c/g543722</t>
@@ -9752,11 +9708,7 @@
       <c r="F247" t="n">
         <v>0</v>
       </c>
-      <c r="G247" t="inlineStr">
-        <is>
-          <t>Cảm biến công nghiệp, Cảm biến lưu lượng</t>
-        </is>
-      </c>
+      <c r="G247" t="inlineStr"/>
       <c r="H247" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/flow-measurement/flow-measurement-instruments/c/g543714</t>
@@ -9790,11 +9742,7 @@
       <c r="F248" t="n">
         <v>0</v>
       </c>
-      <c r="G248" t="inlineStr">
-        <is>
-          <t>Cảm biến công nghiệp, Cảm biến lưu lượng</t>
-        </is>
-      </c>
+      <c r="G248" t="inlineStr"/>
       <c r="H248" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/flow-measurement/flow-metering-systems/c/g472151</t>
@@ -9828,11 +9776,7 @@
       <c r="F249" t="n">
         <v>0</v>
       </c>
-      <c r="G249" t="inlineStr">
-        <is>
-          <t>Cảm biến công nghiệp, Cảm biến lưu lượng</t>
-        </is>
-      </c>
+      <c r="G249" t="inlineStr"/>
       <c r="H249" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/flow-measurement/flow-meters/c/g543715</t>
@@ -10512,11 +10456,7 @@
       <c r="F267" t="n">
         <v>9</v>
       </c>
-      <c r="G267" t="inlineStr">
-        <is>
-          <t>Cảm biến công nghiệp, Cảm biến radar</t>
-        </is>
-      </c>
+      <c r="G267" t="inlineStr"/>
       <c r="H267" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/lidar-and-radar-sensors/radar-sensors/rms/c/g628337</t>
@@ -11196,11 +11136,7 @@
       <c r="F285" t="n">
         <v>2</v>
       </c>
-      <c r="G285" t="inlineStr">
-        <is>
-          <t>Vision và Nhận dạng, Máy đọc mã vạch</t>
-        </is>
-      </c>
+      <c r="G285" t="inlineStr"/>
       <c r="H285" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/machine-vision-and-identification/image-based-code-readers/sensingcam-sec200/c/g625244</t>
@@ -13590,11 +13526,7 @@
       <c r="F348" t="n">
         <v>4</v>
       </c>
-      <c r="G348" t="inlineStr">
-        <is>
-          <t>Encoder bộ mã hóa vòng quay</t>
-        </is>
-      </c>
+      <c r="G348" t="inlineStr"/>
       <c r="H348" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/motion-control-sensors/motor-feedback-systems/ensenm35/c/g623175</t>
@@ -14274,11 +14206,7 @@
       <c r="F366" t="n">
         <v>56</v>
       </c>
-      <c r="G366" t="inlineStr">
-        <is>
-          <t>Bộ kết nối mạng công nghiệp, Đầu nối và cáp</t>
-        </is>
-      </c>
+      <c r="G366" t="inlineStr"/>
       <c r="H366" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/network-and-connection-technology/connectors-and-cables/power-cables/c/g628391</t>
@@ -15638,11 +15566,7 @@
       <c r="F402" t="n">
         <v>0</v>
       </c>
-      <c r="G402" t="inlineStr">
-        <is>
-          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
-        </is>
-      </c>
+      <c r="G402" t="inlineStr"/>
       <c r="H402" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/other-products/c/g575324</t>
@@ -19402,7 +19326,7 @@
       </c>
       <c r="G501" t="inlineStr">
         <is>
-          <t>Thiết bị an toàn máy, Công tắc an toàn</t>
+          <t>Cảm biến công nghiệp, Cảm biến tiệm cận</t>
         </is>
       </c>
       <c r="H501" t="inlineStr">
@@ -19440,7 +19364,7 @@
       </c>
       <c r="G502" t="inlineStr">
         <is>
-          <t>Thiết bị an toàn máy, Công tắc an toàn</t>
+          <t>Cảm biến công nghiệp, Cảm biến tiệm cận</t>
         </is>
       </c>
       <c r="H502" t="inlineStr">
@@ -19516,7 +19440,7 @@
       </c>
       <c r="G504" t="inlineStr">
         <is>
-          <t>Thiết bị an toàn máy, Công tắc an toàn</t>
+          <t>Cảm biến công nghiệp, Cảm biến tiệm cận</t>
         </is>
       </c>
       <c r="H504" t="inlineStr">
@@ -20808,7 +20732,7 @@
       </c>
       <c r="G538" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Camera công nghiệp 2D/3D</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H538" t="inlineStr">
@@ -20920,11 +20844,7 @@
       <c r="F541" t="n">
         <v>1</v>
       </c>
-      <c r="G541" t="inlineStr">
-        <is>
-          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
-        </is>
-      </c>
+      <c r="G541" t="inlineStr"/>
       <c r="H541" t="inlineStr">
         <is>
           <t>https://www.sick.com/sg/en/catalog/products/systems/quality-control-systems/pallet-serialization-system/c/g624914</t>
@@ -21036,7 +20956,7 @@
       </c>
       <c r="G544" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Camera công nghiệp 2D/3D</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H544" t="inlineStr">
@@ -21074,7 +20994,7 @@
       </c>
       <c r="G545" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Camera công nghiệp 2D/3D</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H545" t="inlineStr">
@@ -21112,7 +21032,7 @@
       </c>
       <c r="G546" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Camera công nghiệp 2D/3D</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H546" t="inlineStr">
@@ -21150,7 +21070,7 @@
       </c>
       <c r="G547" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Máy đọc mã vạch</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H547" t="inlineStr">
@@ -21264,7 +21184,7 @@
       </c>
       <c r="G550" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Camera công nghiệp 2D/3D</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H550" t="inlineStr">
@@ -21302,7 +21222,7 @@
       </c>
       <c r="G551" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Đầu đọc RFID</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H551" t="inlineStr">
@@ -21378,7 +21298,7 @@
       </c>
       <c r="G553" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Camera công nghiệp 2D/3D</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H553" t="inlineStr">
@@ -21416,7 +21336,7 @@
       </c>
       <c r="G554" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Camera công nghiệp 2D/3D</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H554" t="inlineStr">
@@ -21530,7 +21450,7 @@
       </c>
       <c r="G557" t="inlineStr">
         <is>
-          <t>Vision và Nhận dạng, Đầu đọc RFID</t>
+          <t>Không có danh mục sản phẩm,  chỉ nằm trong danh mục Thương Hiệu SICK Sensor</t>
         </is>
       </c>
       <c r="H557" t="inlineStr">

</xml_diff>